<commit_message>
feat: verify rule CG0088 and add negative test cases
</commit_message>
<xml_diff>
--- a/rules/CORE-000015/negative/01/data/unit-test-coreid-CG0088-negative.xlsx
+++ b/rules/CORE-000015/negative/01/data/unit-test-coreid-CG0088-negative.xlsx
@@ -1,29 +1,29 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Library" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Datasets" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Validation" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="ag.xpt" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="cm.xpt" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="ec.xpt" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="ex.xpt" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="ml.xpt" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="pr.xpt" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="su.xpt" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="ae.xpt" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="be.xpt" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="ce.xpt" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet name="ds.xpt" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet name="dv.xpt" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet name="ho.xpt" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet name="mh.xpt" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Library" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Datasets" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Validation" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ag.xpt" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="cm.xpt" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ec.xpt" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ex.xpt" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ml.xpt" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pr.xpt" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="su.xpt" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ae.xpt" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="be.xpt" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ce.xpt" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ds.xpt" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="dv.xpt" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ho.xpt" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="mh.xpt" sheetId="17" state="visible" r:id="rId17"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -48,7 +48,7 @@
       <i val="1"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -59,6 +59,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="00FFFFCC"/>
         <bgColor rgb="00FFFFCC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor rgb="FFFFFF00"/>
       </patternFill>
     </fill>
   </fills>
@@ -104,7 +110,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -123,6 +129,12 @@
       <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="2" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -557,7 +569,7 @@
           <t>SUTRT</t>
         </is>
       </c>
-      <c r="F1" s="2" t="inlineStr">
+      <c r="F1" s="8" t="inlineStr">
         <is>
           <t>SUOCCUR</t>
         </is>
@@ -952,7 +964,7 @@
           <t>BETERM</t>
         </is>
       </c>
-      <c r="F1" s="2" t="inlineStr">
+      <c r="F1" s="8" t="inlineStr">
         <is>
           <t>BEOCCUR</t>
         </is>
@@ -1186,7 +1198,7 @@
           <t>CETERM</t>
         </is>
       </c>
-      <c r="F1" s="2" t="inlineStr">
+      <c r="F1" s="8" t="inlineStr">
         <is>
           <t>CEOCCUR</t>
         </is>
@@ -1986,7 +1998,7 @@
           <t>HOTERM</t>
         </is>
       </c>
-      <c r="F1" s="2" t="inlineStr">
+      <c r="F1" s="8" t="inlineStr">
         <is>
           <t>HOOCCUR</t>
         </is>
@@ -2216,7 +2228,7 @@
           <t>MHTERM</t>
         </is>
       </c>
-      <c r="F1" s="2" t="inlineStr">
+      <c r="F1" s="8" t="inlineStr">
         <is>
           <t>MHOCCUR</t>
         </is>
@@ -2611,7 +2623,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F1"/>
+  <dimension ref="A1:F21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2643,6 +2655,566 @@
       <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Error value</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>ag.xpt</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Variable</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>AGOCCUR</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>[PRESENT]</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>1</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>ag.xpt</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Variable</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>AGPRESP</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Not in dataset</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>2</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>cm.xpt</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Variable</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>1</v>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>CMOCCUR</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>[PRESENT]</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>2</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>cm.xpt</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Variable</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>1</v>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>CMPRESP</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Not in dataset</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>3</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>ec.xpt</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Variable</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>ECOCCUR</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>[PRESENT]</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>3</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>ec.xpt</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Variable</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>1</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>ECPRESP</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Not in dataset</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>4</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>ml.xpt</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Variable</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>MLOCCUR</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>[PRESENT]</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>4</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>ml.xpt</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Variable</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>1</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>MLPRESP</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Not in dataset</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>5</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>pr.xpt</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Variable</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>1</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>PROCCUR</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>[PRESENT]</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>5</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>pr.xpt</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Variable</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>1</v>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>PRPRESP</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Not in dataset</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>6</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>su.xpt</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Variable</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>1</v>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>SUOCCUR</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>[PRESENT]</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>6</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>su.xpt</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Variable</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>1</v>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>SUPRESP</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Not in dataset</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>7</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>be.xpt</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Variable</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>1</v>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>BEOCCUR</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>[PRESENT]</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>7</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>be.xpt</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Variable</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>1</v>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>BEPRESP</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Not in dataset</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>8</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>ce.xpt</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Variable</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>1</v>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>CEOCCUR</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>[PRESENT]</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>8</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>ce.xpt</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Variable</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>1</v>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>CEPRESP</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Not in dataset</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>9</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>ho.xpt</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Variable</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>1</v>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>HOOCCUR</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>[PRESENT]</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>9</v>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>ho.xpt</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Variable</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>1</v>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>HOPRESP</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>Not in dataset</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>10</v>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>mh.xpt</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Variable</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>1</v>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>MHOCCUR</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>[PRESENT]</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>10</v>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>mh.xpt</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Variable</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>1</v>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>MHPRESP</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>Not in dataset</t>
         </is>
       </c>
     </row>
@@ -2686,7 +3258,7 @@
           <t>AGTRT</t>
         </is>
       </c>
-      <c r="F1" s="2" t="inlineStr">
+      <c r="F1" s="8" t="inlineStr">
         <is>
           <t>AGOCCUR</t>
         </is>
@@ -2891,7 +3463,7 @@
           <t>CMTRT</t>
         </is>
       </c>
-      <c r="F1" s="2" t="inlineStr">
+      <c r="F1" s="8" t="inlineStr">
         <is>
           <t>CMOCCUR</t>
         </is>
@@ -3096,7 +3668,7 @@
           <t>ECTRT</t>
         </is>
       </c>
-      <c r="F1" s="6" t="inlineStr">
+      <c r="F1" s="9" t="inlineStr">
         <is>
           <t>ECOCCUR</t>
         </is>
@@ -3610,7 +4182,7 @@
           <t>MLTRT</t>
         </is>
       </c>
-      <c r="F1" s="2" t="inlineStr">
+      <c r="F1" s="8" t="inlineStr">
         <is>
           <t>MLOCCUR</t>
         </is>
@@ -3815,7 +4387,7 @@
           <t>PRTRT</t>
         </is>
       </c>
-      <c r="F1" s="2" t="inlineStr">
+      <c r="F1" s="8" t="inlineStr">
         <is>
           <t>PROCCUR</t>
         </is>

</xml_diff>